<commit_message>
Update running Excel source with latest activity data
</commit_message>
<xml_diff>
--- a/data/data lari-2026-9-18-9.xlsx
+++ b/data/data lari-2026-9-18-9.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ryskr\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{06BC886A-64E9-4F9F-8CD6-09AC06A00147}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FB376E6D-4450-466E-942D-7B7B1697759F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{C30B81FF-5A49-42E1-B2DD-9886C1675222}"/>
+    <workbookView xWindow="3300" yWindow="2810" windowWidth="12920" windowHeight="7270" xr2:uid="{C30B81FF-5A49-42E1-B2DD-9886C1675222}"/>
   </bookViews>
   <sheets>
     <sheet name="data lari-2026-9-18-9" sheetId="1" r:id="rId1"/>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1083" uniqueCount="301">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1087" uniqueCount="302">
   <si>
     <t>Name</t>
   </si>
@@ -926,6 +926,9 @@
   </si>
   <si>
     <t>0.26</t>
+  </si>
+  <si>
+    <t>10.43</t>
   </si>
 </sst>
 </file>
@@ -1433,7 +1436,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1460,6 +1463,11 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="21" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1815,14 +1823,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{79B84B80-E3CA-4535-881F-F3100F80B9E9}">
-  <dimension ref="A1:H216"/>
+  <dimension ref="A1:H217"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="24.7265625" style="6" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="28.08984375" style="9" customWidth="1"/>
     <col min="3" max="3" width="7.90625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="8.1796875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="4.26953125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="4.26953125" customWidth="1"/>
     <col min="6" max="7" width="8.1796875" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="8.36328125" bestFit="1" customWidth="1"/>
   </cols>
@@ -7439,6 +7447,30 @@
         <v>19</v>
       </c>
     </row>
+    <row r="217" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A217" s="5" t="s">
+        <v>106</v>
+      </c>
+      <c r="B217" s="8" t="s">
+        <v>84</v>
+      </c>
+      <c r="C217" s="10" t="s">
+        <v>301</v>
+      </c>
+      <c r="D217" s="3">
+        <v>0.40902777777777777</v>
+      </c>
+      <c r="E217" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="F217" s="11">
+        <v>7.1099537037037031E-2</v>
+      </c>
+      <c r="G217" s="3">
+        <v>0.40902777777777777</v>
+      </c>
+      <c r="H217" s="12"/>
+    </row>
   </sheetData>
   <autoFilter ref="A1:H1" xr:uid="{79B84B80-E3CA-4535-881F-F3100F80B9E9}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>